<commit_message>
Session 2026-09-21: WO-P400-E9.001 (hub_mcp_launcher.ps1 console-log capture), WO-P400-E9.002 (p020_order_writer.py schemas_ops fix)
</commit_message>
<xml_diff>
--- a/projects/P_010_Current_Market_Posture/data/excel_exports/History Grid (QQQ)_v3.xlsx
+++ b/projects/P_010_Current_Market_Posture/data/excel_exports/History Grid (QQQ)_v3.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
   <si>
     <t>High
 Price</t>
@@ -150,10 +150,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" readingOrder="0"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="13.85546875" customWidth="1"/>
@@ -477,37 +477,37 @@
       <c r="A1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="K1" t="s">
         <v>22</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M1" t="s">
@@ -519,27 +519,27 @@
       <c r="Q1" t="s">
         <v>3</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="L2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="L2" s="2"/>
       <c r="M2" t="s">
         <v>4</v>
       </c>
@@ -561,620 +561,688 @@
       <c r="S2" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="1"/>
-      <c r="U2" s="1"/>
-      <c r="V2" s="1"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="2">
-        <v>46280</v>
+      <c r="A3" s="1">
+        <v>46286</v>
       </c>
       <c r="B3">
-        <v>-3.7257080078125</v>
+        <v>14.1966552734375</v>
       </c>
       <c r="C3">
-        <v>-2.99383544921875</v>
+        <v>9.76019287109375</v>
       </c>
       <c r="D3">
-        <v>-3.34271240234375</v>
+        <v>6.7559814453125</v>
       </c>
       <c r="E3">
-        <v>708.799987792969</v>
+        <v>727.890014648438</v>
       </c>
       <c r="F3">
-        <v>709.529907226563</v>
+        <v>743.219970703125</v>
       </c>
       <c r="G3">
-        <v>703.635009765625</v>
+        <v>727.809997558594</v>
       </c>
       <c r="H3">
-        <v>704.539978027344</v>
+        <v>741.469970703125</v>
       </c>
       <c r="I3">
-        <v>709.766967773438</v>
+        <v>740.774353027344</v>
       </c>
       <c r="J3">
-        <v>701.672119140625</v>
+        <v>734.878662109375</v>
       </c>
       <c r="K3">
-        <v>26425030</v>
+        <v>46730600</v>
       </c>
       <c r="L3">
-        <v>-0.158761158585548</v>
+        <v>1.03837943077087</v>
       </c>
       <c r="M3">
-        <v>31.013391494751</v>
+        <v>9.24417209625244</v>
       </c>
       <c r="N3">
-        <v>72.4249877929688</v>
+        <v>-69.1681289672852</v>
       </c>
       <c r="O3" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P3">
-        <v>-38.3391304016113</v>
+        <v>100</v>
       </c>
       <c r="Q3">
-        <v>708.314331054688</v>
+        <v>727.554565429688</v>
       </c>
       <c r="R3">
-        <v>711.752624511719</v>
+        <v>719.755004882813</v>
       </c>
       <c r="S3">
-        <v>712.636901855469</v>
+        <v>716.292663574219</v>
       </c>
       <c r="T3">
-        <v>0.237060546875</v>
+        <v>-2.44561767578125</v>
       </c>
       <c r="U3">
-        <v>-1.962890625</v>
+        <v>7.06866455078125</v>
       </c>
       <c r="V3">
-        <v>8.0948486328125</v>
+        <v>5.89569091796875</v>
       </c>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="2">
-        <v>46279</v>
+      <c r="A4" s="1">
+        <v>46283</v>
       </c>
       <c r="B4">
-        <v>-3.15728759765625</v>
+        <v>6.609130859375</v>
       </c>
       <c r="C4">
-        <v>-1.351806640625</v>
+        <v>1.921875</v>
       </c>
       <c r="D4">
-        <v>-1.42279052734375</v>
+        <v>0.67431640625</v>
       </c>
       <c r="E4">
-        <v>703.325012207031</v>
+        <v>718.830017089844</v>
       </c>
       <c r="F4">
-        <v>712.950012207031</v>
+        <v>721.72998046875</v>
       </c>
       <c r="G4">
-        <v>702.739990234375</v>
+        <v>715.080017089844</v>
       </c>
       <c r="H4">
-        <v>709.179992675781</v>
+        <v>721.450012207031</v>
       </c>
       <c r="I4">
-        <v>711.493713378906</v>
+        <v>722.234802246094</v>
       </c>
       <c r="J4">
-        <v>704.51416015625</v>
+        <v>717.4169921875</v>
       </c>
       <c r="K4">
-        <v>35218900</v>
+        <v>48478700</v>
       </c>
       <c r="L4">
-        <v>-0.0673304945230484</v>
+        <v>0.336475193500519</v>
       </c>
       <c r="M4">
-        <v>17.9865989685059</v>
+        <v>29.9825191497803</v>
       </c>
       <c r="N4">
-        <v>-36.6665992736816</v>
+        <v>-4.98308420181274</v>
       </c>
       <c r="O4" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P4">
-        <v>-36.0640640258789</v>
+        <v>80.4549713134766</v>
       </c>
       <c r="Q4">
-        <v>711.302185058594</v>
+        <v>716.06591796875</v>
       </c>
       <c r="R4">
-        <v>713.587768554688</v>
+        <v>713.820434570313</v>
       </c>
       <c r="S4">
-        <v>713.460144042969</v>
+        <v>713.369812011719</v>
       </c>
       <c r="T4">
-        <v>-1.456298828125</v>
+        <v>0.50482177734375</v>
       </c>
       <c r="U4">
-        <v>1.774169921875</v>
+        <v>2.33697509765625</v>
       </c>
       <c r="V4">
-        <v>6.97955322265625</v>
+        <v>4.81781005859375</v>
       </c>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="2">
-        <v>46276</v>
+      <c r="A5" s="1">
+        <v>46282</v>
       </c>
       <c r="B5">
-        <v>-1.25286865234375</v>
+        <v>3.13165283203125</v>
       </c>
       <c r="C5">
-        <v>-0.0504150390625</v>
+        <v>-1.364501953125</v>
       </c>
       <c r="D5">
-        <v>0.0614013671875</v>
+        <v>-2.145751953125</v>
       </c>
       <c r="E5">
-        <v>715.679992675781</v>
+        <v>715.950012207031</v>
       </c>
       <c r="F5">
-        <v>717.630004882813</v>
+        <v>718.040100097656</v>
       </c>
       <c r="G5">
-        <v>713.630004882813</v>
+        <v>713.320007324219</v>
       </c>
       <c r="H5">
-        <v>714.880004882813</v>
+        <v>716.919982910156</v>
       </c>
       <c r="I5">
-        <v>717.939086914063</v>
+        <v>719.826782226563</v>
       </c>
       <c r="J5">
-        <v>713.56103515625</v>
+        <v>714.528686523438</v>
       </c>
       <c r="K5">
-        <v>26649100</v>
+        <v>37270200</v>
       </c>
       <c r="L5">
-        <v>-0.0166160948574543</v>
+        <v>0.00647553941234946</v>
       </c>
       <c r="M5">
-        <v>28.3998622894287</v>
+        <v>31.5549278259277</v>
       </c>
       <c r="N5">
-        <v>-15.047513961792</v>
+        <v>-24.4697818756104</v>
       </c>
       <c r="O5" t="s">
         <v>1</v>
       </c>
       <c r="P5">
-        <v>17.6300525665283</v>
+        <v>100</v>
       </c>
       <c r="Q5">
-        <v>714.212158203125</v>
+        <v>711.757141113281</v>
       </c>
       <c r="R5">
-        <v>714.767395019531</v>
+        <v>711.859619140625</v>
       </c>
       <c r="S5">
-        <v>714.118408203125</v>
+        <v>712.403137207031</v>
       </c>
       <c r="T5">
-        <v>0.30908203125</v>
+        <v>1.78668212890625</v>
       </c>
       <c r="U5">
-        <v>-0.0689697265625</v>
+        <v>1.20867919921875</v>
       </c>
       <c r="V5">
-        <v>4.3780517578125</v>
+        <v>5.298095703125</v>
       </c>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="2">
-        <v>46275</v>
+      <c r="A6" s="1">
+        <v>46281</v>
       </c>
       <c r="B6">
-        <v>-4.352294921875</v>
+        <v>-3.04632568359375</v>
       </c>
       <c r="C6">
-        <v>-1.41351318359375</v>
+        <v>-4.61907958984375</v>
       </c>
       <c r="D6">
-        <v>-0.0198974609375</v>
+        <v>-4.482666015625</v>
       </c>
       <c r="E6">
-        <v>707.549987792969</v>
+        <v>708</v>
       </c>
       <c r="F6">
-        <v>712.059997558594</v>
+        <v>711.880004882813</v>
       </c>
       <c r="G6">
-        <v>706.85498046875</v>
+        <v>700</v>
       </c>
       <c r="H6">
-        <v>708.690002441406</v>
+        <v>704.719970703125</v>
       </c>
       <c r="I6">
-        <v>712.571716308594</v>
+        <v>708.136596679688</v>
       </c>
       <c r="J6">
-        <v>705.699035644531</v>
+        <v>700.750732421875</v>
       </c>
       <c r="K6">
-        <v>31414400</v>
+        <v>35687900</v>
       </c>
       <c r="L6">
-        <v>-0.139474049210548</v>
+        <v>-0.168285548686981</v>
       </c>
       <c r="M6">
-        <v>33.430290222168</v>
+        <v>41.7778854370117</v>
       </c>
       <c r="N6">
-        <v>-17.8725566864014</v>
+        <v>34.7091789245605</v>
       </c>
       <c r="O6" t="s">
         <v>23</v>
       </c>
       <c r="P6">
-        <v>-58.667163848877</v>
+        <v>-16.5481777191162</v>
       </c>
       <c r="Q6">
-        <v>712.955444335938</v>
+        <v>706.420654296875</v>
       </c>
       <c r="R6">
-        <v>714.558349609375</v>
+        <v>710.200256347656</v>
       </c>
       <c r="S6">
-        <v>714.115844726563</v>
+        <v>711.805541992188</v>
       </c>
       <c r="T6">
-        <v>0.51171875</v>
+        <v>-3.743408203125</v>
       </c>
       <c r="U6">
-        <v>-1.15594482421875</v>
+        <v>0.750732421875</v>
       </c>
       <c r="V6">
-        <v>6.8726806640625</v>
+        <v>7.3858642578125</v>
       </c>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="2">
-        <v>46274</v>
+      <c r="A7" s="1">
+        <v>46280</v>
       </c>
       <c r="B7">
-        <v>0.855224609375</v>
+        <v>-3.7257080078125</v>
       </c>
       <c r="C7">
-        <v>1.43170166015625</v>
+        <v>-2.99383544921875</v>
       </c>
       <c r="D7">
-        <v>1.8648681640625</v>
+        <v>-3.34271240234375</v>
       </c>
       <c r="E7">
-        <v>716.400024414063</v>
+        <v>708.799987792969</v>
       </c>
       <c r="F7">
-        <v>719.700012207031</v>
+        <v>709.529907226563</v>
       </c>
       <c r="G7">
-        <v>714.02001953125</v>
+        <v>703.635009765625</v>
       </c>
       <c r="H7">
-        <v>716.309997558594</v>
+        <v>704.539978027344</v>
       </c>
       <c r="I7">
-        <v>719.557373046875</v>
+        <v>709.766967773438</v>
       </c>
       <c r="J7">
-        <v>713.248901367188</v>
+        <v>701.672119140625</v>
       </c>
       <c r="K7">
-        <v>26763300</v>
+        <v>26631600</v>
       </c>
       <c r="L7">
-        <v>-0.424235016107559</v>
+        <v>-0.158761158585548</v>
       </c>
       <c r="M7">
-        <v>40.7053833007813</v>
+        <v>31.013391494751</v>
       </c>
       <c r="N7">
-        <v>-8.74598026275635</v>
+        <v>72.4249877929688</v>
       </c>
       <c r="O7" t="s">
         <v>23</v>
       </c>
       <c r="P7">
-        <v>-8.89947319030762</v>
+        <v>-38.3391304016113</v>
       </c>
       <c r="Q7">
-        <v>716.923706054688</v>
+        <v>708.314331054688</v>
       </c>
       <c r="R7">
-        <v>716.138122558594</v>
+        <v>711.752624511719</v>
       </c>
       <c r="S7">
-        <v>714.806884765625</v>
+        <v>712.636901855469</v>
       </c>
       <c r="T7">
-        <v>-0.14263916015625</v>
+        <v>0.237060546875</v>
       </c>
       <c r="U7">
-        <v>-0.7711181640625</v>
+        <v>-1.962890625</v>
       </c>
       <c r="V7">
-        <v>6.3084716796875</v>
+        <v>8.0948486328125</v>
       </c>
     </row>
     <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="2">
-        <v>46273</v>
+      <c r="A8" s="1">
+        <v>46279</v>
       </c>
       <c r="B8">
-        <v>3.77337646484375</v>
+        <v>-3.15728759765625</v>
       </c>
       <c r="C8">
-        <v>2.11810302734375</v>
+        <v>-1.351806640625</v>
       </c>
       <c r="D8">
-        <v>1.7724609375</v>
+        <v>-1.42279052734375</v>
       </c>
       <c r="E8">
-        <v>720.908996582031</v>
+        <v>703.325012207031</v>
       </c>
       <c r="F8">
-        <v>721.885986328125</v>
+        <v>712.950012207031</v>
       </c>
       <c r="G8">
-        <v>715.570007324219</v>
+        <v>702.739990234375</v>
       </c>
       <c r="H8">
-        <v>718.359985351563</v>
+        <v>709.179992675781</v>
       </c>
       <c r="I8">
-        <v>721.029541015625</v>
+        <v>711.493713378906</v>
       </c>
       <c r="J8">
-        <v>715.595031738281</v>
+        <v>704.51416015625</v>
       </c>
       <c r="K8">
-        <v>28341400</v>
+        <v>35218900</v>
       </c>
       <c r="L8">
-        <v>-0.492329925298691</v>
+        <v>-0.0673304945230484</v>
       </c>
       <c r="M8">
-        <v>44.6066741943359</v>
+        <v>17.9865989685059</v>
       </c>
       <c r="N8">
-        <v>-6.65095376968384</v>
+        <v>-36.6665992736816</v>
       </c>
       <c r="O8" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="P8">
-        <v>10.4499626159668</v>
+        <v>-36.0640640258789</v>
       </c>
       <c r="Q8">
-        <v>717.470703125</v>
+        <v>711.302185058594</v>
       </c>
       <c r="R8">
-        <v>715.960205078125</v>
+        <v>713.587768554688</v>
       </c>
       <c r="S8">
-        <v>714.734558105469</v>
+        <v>713.460144042969</v>
       </c>
       <c r="T8">
-        <v>-0.8564453125</v>
+        <v>-1.456298828125</v>
       </c>
       <c r="U8">
-        <v>0.0250244140625</v>
+        <v>1.774169921875</v>
       </c>
       <c r="V8">
-        <v>5.43450927734375</v>
+        <v>6.97955322265625</v>
       </c>
     </row>
     <row r="9" ht="19.5" customHeight="1">
-      <c r="A9" s="2">
-        <v>46269</v>
+      <c r="A9" s="1">
+        <v>46276</v>
       </c>
       <c r="B9">
-        <v>3.72772216796875</v>
+        <v>-1.25286865234375</v>
       </c>
       <c r="C9">
-        <v>2.60296630859375</v>
+        <v>-0.0504150390625</v>
       </c>
       <c r="D9">
-        <v>0.3096923828125</v>
+        <v>0.0614013671875</v>
       </c>
       <c r="E9">
-        <v>719.340026855469</v>
+        <v>715.679992675781</v>
       </c>
       <c r="F9">
-        <v>721.859985351563</v>
+        <v>717.630004882813</v>
       </c>
       <c r="G9">
-        <v>716.559997558594</v>
+        <v>713.630004882813</v>
       </c>
       <c r="H9">
-        <v>718.960021972656</v>
+        <v>714.880004882813</v>
       </c>
       <c r="I9">
-        <v>722.363159179688</v>
+        <v>717.939086914063</v>
       </c>
       <c r="J9">
-        <v>716.705444335938</v>
+        <v>713.56103515625</v>
       </c>
       <c r="K9">
-        <v>32871000</v>
+        <v>26649100</v>
       </c>
       <c r="L9">
-        <v>-0.23380534350872</v>
+        <v>-0.0166160948574543</v>
       </c>
       <c r="M9">
-        <v>47.7848205566406</v>
+        <v>28.3998622894287</v>
       </c>
       <c r="N9">
-        <v>-7.74872875213623</v>
+        <v>-15.047513961792</v>
       </c>
       <c r="O9" t="s">
         <v>1</v>
       </c>
       <c r="P9">
-        <v>57.7196006774902</v>
+        <v>17.6300525665283</v>
       </c>
       <c r="Q9">
-        <v>716.620361328125</v>
+        <v>714.212158203125</v>
       </c>
       <c r="R9">
-        <v>715.381286621094</v>
+        <v>714.767395019531</v>
       </c>
       <c r="S9">
-        <v>714.463317871094</v>
+        <v>714.118408203125</v>
       </c>
       <c r="T9">
-        <v>0.503173828125</v>
+        <v>0.30908203125</v>
       </c>
       <c r="U9">
-        <v>0.14544677734375</v>
+        <v>-0.0689697265625</v>
       </c>
       <c r="V9">
-        <v>5.65771484375</v>
+        <v>4.3780517578125</v>
       </c>
     </row>
     <row r="10" ht="19.5" customHeight="1">
-      <c r="A10" s="2">
-        <v>46268</v>
+      <c r="A10" s="1">
+        <v>46275</v>
       </c>
       <c r="B10">
-        <v>1.111083984375</v>
+        <v>-4.352294921875</v>
       </c>
       <c r="C10">
-        <v>0.99615478515625</v>
+        <v>-1.41351318359375</v>
       </c>
       <c r="D10">
-        <v>-2.15606689453125</v>
+        <v>-0.0198974609375</v>
       </c>
       <c r="E10">
-        <v>710.849975585938</v>
+        <v>707.549987792969</v>
       </c>
       <c r="F10">
-        <v>718.914978027344</v>
+        <v>712.059997558594</v>
       </c>
       <c r="G10">
-        <v>709.690002441406</v>
+        <v>706.85498046875</v>
       </c>
       <c r="H10">
-        <v>717.669982910156</v>
+        <v>708.690002441406</v>
       </c>
       <c r="I10">
-        <v>719.351440429688</v>
+        <v>712.571716308594</v>
       </c>
       <c r="J10">
-        <v>714.108703613281</v>
+        <v>705.699035644531</v>
       </c>
       <c r="K10">
-        <v>29449700</v>
+        <v>31414400</v>
       </c>
       <c r="L10">
-        <v>-0.0333281010389328</v>
+        <v>-0.139474049210548</v>
       </c>
       <c r="M10">
-        <v>51.7985496520996</v>
+        <v>33.430290222168</v>
       </c>
       <c r="N10">
-        <v>-23.523889541626</v>
+        <v>-17.8725566864014</v>
       </c>
       <c r="O10" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="P10">
-        <v>50.7881851196289</v>
+        <v>-58.667163848877</v>
       </c>
       <c r="Q10">
-        <v>713.895751953125</v>
+        <v>712.955444335938</v>
       </c>
       <c r="R10">
-        <v>714.236145019531</v>
+        <v>714.558349609375</v>
       </c>
       <c r="S10">
-        <v>713.808471679688</v>
+        <v>714.115844726563</v>
       </c>
       <c r="T10">
-        <v>0.43646240234375</v>
+        <v>0.51171875</v>
       </c>
       <c r="U10">
-        <v>4.418701171875</v>
+        <v>-1.15594482421875</v>
       </c>
       <c r="V10">
-        <v>5.24273681640625</v>
+        <v>6.8726806640625</v>
       </c>
     </row>
     <row r="11" ht="19.5" customHeight="1">
-      <c r="A11" s="2">
-        <v>46267</v>
+      <c r="A11" s="1">
+        <v>46274</v>
       </c>
       <c r="B11">
-        <v>-4.34771728515625</v>
+        <v>0.855224609375</v>
       </c>
       <c r="C11">
-        <v>-0.8651123046875</v>
+        <v>1.43170166015625</v>
       </c>
       <c r="D11">
-        <v>-4.5257568359375</v>
+        <v>1.8648681640625</v>
       </c>
       <c r="E11">
-        <v>707.099975585938</v>
+        <v>716.400024414063</v>
       </c>
       <c r="F11">
-        <v>709.798889160156</v>
+        <v>719.700012207031</v>
       </c>
       <c r="G11">
-        <v>705.099975585938</v>
+        <v>714.02001953125</v>
       </c>
       <c r="H11">
-        <v>709.239990234375</v>
+        <v>716.309997558594</v>
       </c>
       <c r="I11">
-        <v>712.845642089844</v>
+        <v>719.557373046875</v>
       </c>
       <c r="J11">
-        <v>706.473327636719</v>
+        <v>713.248901367188</v>
       </c>
       <c r="K11">
-        <v>23476200</v>
+        <v>26763300</v>
       </c>
       <c r="L11">
-        <v>-0.784281432628632</v>
+        <v>-0.424235016107559</v>
       </c>
       <c r="M11">
-        <v>67.7316741943359</v>
+        <v>40.7053833007813</v>
       </c>
       <c r="N11">
-        <v>-9.31163692474365</v>
+        <v>-8.74598026275635</v>
       </c>
       <c r="O11" t="s">
         <v>23</v>
       </c>
       <c r="P11">
-        <v>-10.4177856445313</v>
+        <v>-8.89947319030762</v>
       </c>
       <c r="Q11">
-        <v>710.752807617188</v>
+        <v>716.923706054688</v>
       </c>
       <c r="R11">
-        <v>713.091125488281</v>
+        <v>716.138122558594</v>
       </c>
       <c r="S11">
-        <v>713.333984375</v>
+        <v>714.806884765625</v>
       </c>
       <c r="T11">
-        <v>3.0467529296875</v>
+        <v>-0.14263916015625</v>
       </c>
       <c r="U11">
-        <v>1.37335205078125</v>
+        <v>-0.7711181640625</v>
       </c>
       <c r="V11">
-        <v>6.372314453125</v>
+        <v>6.3084716796875</v>
+      </c>
+    </row>
+    <row r="12" ht="19.5" customHeight="1">
+      <c r="A12" s="1">
+        <v>46273</v>
+      </c>
+      <c r="B12">
+        <v>3.77337646484375</v>
+      </c>
+      <c r="C12">
+        <v>2.11810302734375</v>
+      </c>
+      <c r="D12">
+        <v>1.7724609375</v>
+      </c>
+      <c r="E12">
+        <v>720.908996582031</v>
+      </c>
+      <c r="F12">
+        <v>721.885986328125</v>
+      </c>
+      <c r="G12">
+        <v>715.570007324219</v>
+      </c>
+      <c r="H12">
+        <v>718.359985351563</v>
+      </c>
+      <c r="I12">
+        <v>721.029541015625</v>
+      </c>
+      <c r="J12">
+        <v>715.595031738281</v>
+      </c>
+      <c r="K12">
+        <v>28341400</v>
+      </c>
+      <c r="L12">
+        <v>-0.492329925298691</v>
+      </c>
+      <c r="M12">
+        <v>44.6066741943359</v>
+      </c>
+      <c r="N12">
+        <v>-6.65095376968384</v>
+      </c>
+      <c r="O12" t="s">
+        <v>1</v>
+      </c>
+      <c r="P12">
+        <v>10.4499626159668</v>
+      </c>
+      <c r="Q12">
+        <v>717.470703125</v>
+      </c>
+      <c r="R12">
+        <v>715.960205078125</v>
+      </c>
+      <c r="S12">
+        <v>714.734558105469</v>
+      </c>
+      <c r="T12">
+        <v>-0.8564453125</v>
+      </c>
+      <c r="U12">
+        <v>0.0250244140625</v>
+      </c>
+      <c r="V12">
+        <v>5.43450927734375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>